<commit_message>
fix: rewrite patterns for fixtures 18-22 with correct cell layout
All five MS-template fixture patterns were rewritten from scratch to
match the actual cell layout of the restored data files:

- F18 billing_statement: absolute KV cells (C8,F8,C9,C10) + transaction table
- F19 blood_pressure_tracker: absolute target cells (D7,E7) + readings table
- F20 sales_report: correct lbl headers ('Summe aus Qrtl 1' etc.)
- F21 monthly_budget: absolute KV cells + IGNORE-anchored expense tables
  capturing category names in column B
- F22 weekly_timesheet: absolute KV cells; single week table:* finds both
  week blocks naturally; pay section uses absolute cells (H30:L31) to avoid
  FOOTER ambiguity; col_breaks regex escapes literal parens \(minutes\)

989 passed, 3 xfailed in test suite.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/19_blood_pressure_tracker/pattern.xlsx
+++ b/tests/fixtures/19_blood_pressure_tracker/pattern.xlsx
@@ -413,30 +413,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>```</t>
+          <t>config:</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>read.direction</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>LR</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>config:</t>
+          <t>lbl:</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>read.direction</t>
+          <t>col_datum</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LR</t>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Datum</t>
         </is>
       </c>
     </row>
@@ -448,7 +463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>lbl_blutdruckerfassung</t>
+          <t>col_zeit</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -458,7 +473,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Blutdruckerfassung</t>
+          <t>Zeit</t>
         </is>
       </c>
     </row>
@@ -470,7 +485,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>lbl_name</t>
+          <t>col_systolisch</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -480,7 +495,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Systolisch</t>
         </is>
       </c>
     </row>
@@ -492,7 +507,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>col_systolisch</t>
+          <t>col_diastolisch</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -502,7 +517,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Systolisch</t>
+          <t>Diastolisch</t>
         </is>
       </c>
     </row>
@@ -514,7 +529,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>col_diastolisch</t>
+          <t>col_herzfrequenz</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -524,7 +539,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Diastolisch</t>
+          <t>Herzfrequenz</t>
         </is>
       </c>
     </row>
@@ -536,7 +551,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>lbl_telefon</t>
+          <t>col_kommentare</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -546,85 +561,81 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Telefonnummer des behandelnden Arztes</t>
+          <t>Kommentare</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>lbl:</t>
+          <t>var:</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>lbl_standard</t>
+          <t>target.systolic</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>\*\ Standard\ des\ Gesundheitsministeriums</t>
+          <t>\d+</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>lbl:</t>
+          <t>var:</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>lbl_datum</t>
+          <t>target.diastolic</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>\d+</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>lbl:</t>
+          <t>var:</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>lbl_systolisch</t>
+          <t>measurement.date</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Systolisch</t>
-        </is>
-      </c>
+          <t>datetime</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>lbl:</t>
+          <t>var:</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>lbl_herzfrequenz</t>
+          <t>measurement.time</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -634,51 +645,51 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Herzfrequenz</t>
+          <t>.*</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>lbl:</t>
+          <t>var:</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>lbl_zeit</t>
+          <t>measurement.systolic</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Zeit</t>
+          <t>\d+</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lbl:</t>
+          <t>var:</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>lbl_kommentare</t>
+          <t>measurement.diastolic</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Kommentare</t>
+          <t>\d+</t>
         </is>
       </c>
     </row>
@@ -690,12 +701,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>measurement.date</t>
+          <t>measurement.heart_rate</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>\d+</t>
         </is>
       </c>
     </row>
@@ -707,7 +723,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>measurement.time</t>
+          <t>measurement.comments</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -724,440 +740,119 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>measurement.systolic</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>\d+</t>
+          <t>START:</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>var:</t>
+          <t>cell:D7</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>measurement.diastolic</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>\d+</t>
+          <t>target.systolic</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>var:</t>
+          <t>cell:E7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>measurement.heart_rate</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>\d+</t>
+          <t>target.diastolic</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>var:</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+          <t>table:*</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HEADER:1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>col_datum</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>col_zeit</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>col_systolisch</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>col_diastolisch</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>col_herzfrequenz</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>col_kommentare</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DATA:*</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>measurement.date</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>measurement.time</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>measurement.systolic</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>measurement.diastolic</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>measurement.heart_rate</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>measurement.comments</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>.*</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>START:</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>lbl_blutdruckerfassung</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>lbl_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>table:*</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>col_systolisch</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>col_diastolisch</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>DATA:1</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>measurement.systolic</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>measurement.diastolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>table:*</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>col_systolisch</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>col_diastolisch</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>DATA:1</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>lbl_telefon</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>lbl_standard</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>IGNORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>lbl_datum</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>lbl_zeit</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>lbl_systolisch</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>col_diastolisch</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>lbl_herzfrequenz</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>cell:next</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>lbl_kommentare</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>table:*</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>HEADER:1</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>lbl_datum</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>lbl_zeit</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>lbl_systolisch</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>col_diastolisch</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>lbl_herzfrequenz</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>lbl_kommentare</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>DATA:*</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>measurement.date</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>measurement.time</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>measurement.systolic</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>measurement.diastolic</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>measurement.heart_rate</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>measurement.comments</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
           <t>END:</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>```</t>
         </is>
       </c>
     </row>

</xml_diff>